<commit_message>
Fixed Fairfax Geocoding and Download
</commit_message>
<xml_diff>
--- a/wateruse.xlsx
+++ b/wateruse.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4015" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3958" uniqueCount="52">
   <si>
     <t>Company</t>
   </si>
@@ -170,150 +170,6 @@
   </si>
   <si>
     <t>13600 Eds Dr</t>
-  </si>
-  <si>
-    <t>2023-03-01</t>
-  </si>
-  <si>
-    <t>2025-11-14</t>
-  </si>
-  <si>
-    <t>2023-02-03</t>
-  </si>
-  <si>
-    <t>2023-05-01</t>
-  </si>
-  <si>
-    <t>2023-08-01</t>
-  </si>
-  <si>
-    <t>2023-10-31</t>
-  </si>
-  <si>
-    <t>2024-02-01</t>
-  </si>
-  <si>
-    <t>2024-05-01</t>
-  </si>
-  <si>
-    <t>2024-07-30</t>
-  </si>
-  <si>
-    <t>2024-11-01</t>
-  </si>
-  <si>
-    <t>2025-02-03</t>
-  </si>
-  <si>
-    <t>2025-05-05</t>
-  </si>
-  <si>
-    <t>2025-07-31</t>
-  </si>
-  <si>
-    <t>2025-10-29</t>
-  </si>
-  <si>
-    <t>2026-01-30</t>
-  </si>
-  <si>
-    <t>2024-04-30</t>
-  </si>
-  <si>
-    <t>2025-01-27</t>
-  </si>
-  <si>
-    <t>2023-07-24</t>
-  </si>
-  <si>
-    <t>2023-10-20</t>
-  </si>
-  <si>
-    <t>2024-01-22</t>
-  </si>
-  <si>
-    <t>2024-04-18</t>
-  </si>
-  <si>
-    <t>2024-07-22</t>
-  </si>
-  <si>
-    <t>2024-10-22</t>
-  </si>
-  <si>
-    <t>2025-01-28</t>
-  </si>
-  <si>
-    <t>2025-04-21</t>
-  </si>
-  <si>
-    <t>2025-07-22</t>
-  </si>
-  <si>
-    <t>2025-10-23</t>
-  </si>
-  <si>
-    <t>2026-01-20</t>
-  </si>
-  <si>
-    <t>2023-05-04</t>
-  </si>
-  <si>
-    <t>2023-08-08</t>
-  </si>
-  <si>
-    <t>2023-09-28</t>
-  </si>
-  <si>
-    <t>2023-11-02</t>
-  </si>
-  <si>
-    <t>2024-02-02</t>
-  </si>
-  <si>
-    <t>2024-05-06</t>
-  </si>
-  <si>
-    <t>2024-08-02</t>
-  </si>
-  <si>
-    <t>2024-11-04</t>
-  </si>
-  <si>
-    <t>2025-02-07</t>
-  </si>
-  <si>
-    <t>2025-05-02</t>
-  </si>
-  <si>
-    <t>2025-08-05</t>
-  </si>
-  <si>
-    <t>2025-11-04</t>
-  </si>
-  <si>
-    <t>2026-02-06</t>
-  </si>
-  <si>
-    <t>2024-06-21</t>
-  </si>
-  <si>
-    <t>2024-09-23</t>
-  </si>
-  <si>
-    <t>2024-12-19</t>
-  </si>
-  <si>
-    <t>2025-03-20</t>
-  </si>
-  <si>
-    <t>2025-06-18</t>
-  </si>
-  <si>
-    <t>2025-09-19</t>
-  </si>
-  <si>
-    <t>2025-12-23</t>
   </si>
 </sst>
 </file>
@@ -22131,8 +21987,8 @@
       <c r="C1262" t="s">
         <v>45</v>
       </c>
-      <c r="D1262" t="s">
-        <v>52</v>
+      <c r="D1262" s="2">
+        <v>44986</v>
       </c>
       <c r="E1262">
         <v>2131000</v>
@@ -22148,8 +22004,8 @@
       <c r="C1263" t="s">
         <v>46</v>
       </c>
-      <c r="D1263" t="s">
-        <v>52</v>
+      <c r="D1263" s="2">
+        <v>44986</v>
       </c>
       <c r="E1263">
         <v>1000</v>
@@ -22165,8 +22021,8 @@
       <c r="C1264" t="s">
         <v>46</v>
       </c>
-      <c r="D1264" t="s">
-        <v>53</v>
+      <c r="D1264" s="2">
+        <v>45975</v>
       </c>
       <c r="E1264">
         <v>0</v>
@@ -22182,8 +22038,8 @@
       <c r="C1265" t="s">
         <v>47</v>
       </c>
-      <c r="D1265" t="s">
-        <v>54</v>
+      <c r="D1265" s="2">
+        <v>44960</v>
       </c>
       <c r="E1265">
         <v>193000</v>
@@ -22199,8 +22055,8 @@
       <c r="C1266" t="s">
         <v>47</v>
       </c>
-      <c r="D1266" t="s">
-        <v>55</v>
+      <c r="D1266" s="2">
+        <v>45047</v>
       </c>
       <c r="E1266">
         <v>573000</v>
@@ -22216,8 +22072,8 @@
       <c r="C1267" t="s">
         <v>47</v>
       </c>
-      <c r="D1267" t="s">
-        <v>56</v>
+      <c r="D1267" s="2">
+        <v>45139</v>
       </c>
       <c r="E1267">
         <v>3694000</v>
@@ -22233,8 +22089,8 @@
       <c r="C1268" t="s">
         <v>47</v>
       </c>
-      <c r="D1268" t="s">
-        <v>57</v>
+      <c r="D1268" s="2">
+        <v>45230</v>
       </c>
       <c r="E1268">
         <v>3083000</v>
@@ -22250,8 +22106,8 @@
       <c r="C1269" t="s">
         <v>47</v>
       </c>
-      <c r="D1269" t="s">
-        <v>58</v>
+      <c r="D1269" s="2">
+        <v>45323</v>
       </c>
       <c r="E1269">
         <v>129000</v>
@@ -22267,8 +22123,8 @@
       <c r="C1270" t="s">
         <v>47</v>
       </c>
-      <c r="D1270" t="s">
-        <v>59</v>
+      <c r="D1270" s="2">
+        <v>45413</v>
       </c>
       <c r="E1270">
         <v>933000</v>
@@ -22284,8 +22140,8 @@
       <c r="C1271" t="s">
         <v>47</v>
       </c>
-      <c r="D1271" t="s">
-        <v>60</v>
+      <c r="D1271" s="2">
+        <v>45503</v>
       </c>
       <c r="E1271">
         <v>7682000</v>
@@ -22301,8 +22157,8 @@
       <c r="C1272" t="s">
         <v>47</v>
       </c>
-      <c r="D1272" t="s">
-        <v>61</v>
+      <c r="D1272" s="2">
+        <v>45597</v>
       </c>
       <c r="E1272">
         <v>4296000</v>
@@ -22318,8 +22174,8 @@
       <c r="C1273" t="s">
         <v>47</v>
       </c>
-      <c r="D1273" t="s">
-        <v>62</v>
+      <c r="D1273" s="2">
+        <v>45691</v>
       </c>
       <c r="E1273">
         <v>157000</v>
@@ -22335,8 +22191,8 @@
       <c r="C1274" t="s">
         <v>47</v>
       </c>
-      <c r="D1274" t="s">
-        <v>63</v>
+      <c r="D1274" s="2">
+        <v>45782</v>
       </c>
       <c r="E1274">
         <v>988000</v>
@@ -22352,8 +22208,8 @@
       <c r="C1275" t="s">
         <v>47</v>
       </c>
-      <c r="D1275" t="s">
-        <v>64</v>
+      <c r="D1275" s="2">
+        <v>45869</v>
       </c>
       <c r="E1275">
         <v>4623000</v>
@@ -22369,8 +22225,8 @@
       <c r="C1276" t="s">
         <v>47</v>
       </c>
-      <c r="D1276" t="s">
-        <v>65</v>
+      <c r="D1276" s="2">
+        <v>45959</v>
       </c>
       <c r="E1276">
         <v>3294000</v>
@@ -22386,8 +22242,8 @@
       <c r="C1277" t="s">
         <v>47</v>
       </c>
-      <c r="D1277" t="s">
-        <v>66</v>
+      <c r="D1277" s="2">
+        <v>46052</v>
       </c>
       <c r="E1277">
         <v>166000</v>
@@ -22403,8 +22259,8 @@
       <c r="C1278" t="s">
         <v>48</v>
       </c>
-      <c r="D1278" t="s">
-        <v>54</v>
+      <c r="D1278" s="2">
+        <v>44960</v>
       </c>
       <c r="E1278">
         <v>8000</v>
@@ -22420,8 +22276,8 @@
       <c r="C1279" t="s">
         <v>48</v>
       </c>
-      <c r="D1279" t="s">
-        <v>55</v>
+      <c r="D1279" s="2">
+        <v>45047</v>
       </c>
       <c r="E1279">
         <v>7000</v>
@@ -22437,8 +22293,8 @@
       <c r="C1280" t="s">
         <v>48</v>
       </c>
-      <c r="D1280" t="s">
-        <v>56</v>
+      <c r="D1280" s="2">
+        <v>45139</v>
       </c>
       <c r="E1280">
         <v>7000</v>
@@ -22454,8 +22310,8 @@
       <c r="C1281" t="s">
         <v>48</v>
       </c>
-      <c r="D1281" t="s">
-        <v>57</v>
+      <c r="D1281" s="2">
+        <v>45230</v>
       </c>
       <c r="E1281">
         <v>7000</v>
@@ -22471,8 +22327,8 @@
       <c r="C1282" t="s">
         <v>48</v>
       </c>
-      <c r="D1282" t="s">
-        <v>58</v>
+      <c r="D1282" s="2">
+        <v>45323</v>
       </c>
       <c r="E1282">
         <v>10000</v>
@@ -22488,8 +22344,8 @@
       <c r="C1283" t="s">
         <v>48</v>
       </c>
-      <c r="D1283" t="s">
-        <v>67</v>
+      <c r="D1283" s="2">
+        <v>45412</v>
       </c>
       <c r="E1283">
         <v>54000</v>
@@ -22505,8 +22361,8 @@
       <c r="C1284" t="s">
         <v>48</v>
       </c>
-      <c r="D1284" t="s">
-        <v>60</v>
+      <c r="D1284" s="2">
+        <v>45503</v>
       </c>
       <c r="E1284">
         <v>56000</v>
@@ -22522,8 +22378,8 @@
       <c r="C1285" t="s">
         <v>48</v>
       </c>
-      <c r="D1285" t="s">
-        <v>61</v>
+      <c r="D1285" s="2">
+        <v>45597</v>
       </c>
       <c r="E1285">
         <v>53000</v>
@@ -22539,8 +22395,8 @@
       <c r="C1286" t="s">
         <v>48</v>
       </c>
-      <c r="D1286" t="s">
-        <v>68</v>
+      <c r="D1286" s="2">
+        <v>45684</v>
       </c>
       <c r="E1286">
         <v>0</v>
@@ -22556,8 +22412,8 @@
       <c r="C1287" t="s">
         <v>49</v>
       </c>
-      <c r="D1287" t="s">
-        <v>69</v>
+      <c r="D1287" s="2">
+        <v>45131</v>
       </c>
       <c r="E1287">
         <v>12000</v>
@@ -22573,8 +22429,8 @@
       <c r="C1288" t="s">
         <v>49</v>
       </c>
-      <c r="D1288" t="s">
-        <v>70</v>
+      <c r="D1288" s="2">
+        <v>45219</v>
       </c>
       <c r="E1288">
         <v>22000</v>
@@ -22590,8 +22446,8 @@
       <c r="C1289" t="s">
         <v>49</v>
       </c>
-      <c r="D1289" t="s">
-        <v>71</v>
+      <c r="D1289" s="2">
+        <v>45313</v>
       </c>
       <c r="E1289">
         <v>32000</v>
@@ -22607,8 +22463,8 @@
       <c r="C1290" t="s">
         <v>49</v>
       </c>
-      <c r="D1290" t="s">
-        <v>72</v>
+      <c r="D1290" s="2">
+        <v>45400</v>
       </c>
       <c r="E1290">
         <v>26000</v>
@@ -22624,8 +22480,8 @@
       <c r="C1291" t="s">
         <v>49</v>
       </c>
-      <c r="D1291" t="s">
-        <v>73</v>
+      <c r="D1291" s="2">
+        <v>45495</v>
       </c>
       <c r="E1291">
         <v>21000</v>
@@ -22641,8 +22497,8 @@
       <c r="C1292" t="s">
         <v>49</v>
       </c>
-      <c r="D1292" t="s">
-        <v>74</v>
+      <c r="D1292" s="2">
+        <v>45587</v>
       </c>
       <c r="E1292">
         <v>19000</v>
@@ -22658,8 +22514,8 @@
       <c r="C1293" t="s">
         <v>49</v>
       </c>
-      <c r="D1293" t="s">
-        <v>75</v>
+      <c r="D1293" s="2">
+        <v>45685</v>
       </c>
       <c r="E1293">
         <v>24000</v>
@@ -22675,8 +22531,8 @@
       <c r="C1294" t="s">
         <v>49</v>
       </c>
-      <c r="D1294" t="s">
-        <v>76</v>
+      <c r="D1294" s="2">
+        <v>45768</v>
       </c>
       <c r="E1294">
         <v>18000</v>
@@ -22692,8 +22548,8 @@
       <c r="C1295" t="s">
         <v>49</v>
       </c>
-      <c r="D1295" t="s">
-        <v>77</v>
+      <c r="D1295" s="2">
+        <v>45860</v>
       </c>
       <c r="E1295">
         <v>22000</v>
@@ -22709,8 +22565,8 @@
       <c r="C1296" t="s">
         <v>49</v>
       </c>
-      <c r="D1296" t="s">
-        <v>78</v>
+      <c r="D1296" s="2">
+        <v>45953</v>
       </c>
       <c r="E1296">
         <v>27000</v>
@@ -22726,8 +22582,8 @@
       <c r="C1297" t="s">
         <v>49</v>
       </c>
-      <c r="D1297" t="s">
-        <v>79</v>
+      <c r="D1297" s="2">
+        <v>46042</v>
       </c>
       <c r="E1297">
         <v>23000</v>
@@ -22743,8 +22599,8 @@
       <c r="C1298" t="s">
         <v>50</v>
       </c>
-      <c r="D1298" t="s">
-        <v>54</v>
+      <c r="D1298" s="2">
+        <v>44960</v>
       </c>
       <c r="E1298">
         <v>360000</v>
@@ -22760,8 +22616,8 @@
       <c r="C1299" t="s">
         <v>50</v>
       </c>
-      <c r="D1299" t="s">
-        <v>80</v>
+      <c r="D1299" s="2">
+        <v>45050</v>
       </c>
       <c r="E1299">
         <v>211000</v>
@@ -22777,8 +22633,8 @@
       <c r="C1300" t="s">
         <v>50</v>
       </c>
-      <c r="D1300" t="s">
-        <v>81</v>
+      <c r="D1300" s="2">
+        <v>45146</v>
       </c>
       <c r="E1300">
         <v>3455000</v>
@@ -22794,8 +22650,8 @@
       <c r="C1301" t="s">
         <v>50</v>
       </c>
-      <c r="D1301" t="s">
-        <v>82</v>
+      <c r="D1301" s="2">
+        <v>45197</v>
       </c>
       <c r="E1301">
         <v>334000</v>
@@ -22811,8 +22667,8 @@
       <c r="C1302" t="s">
         <v>50</v>
       </c>
-      <c r="D1302" t="s">
-        <v>83</v>
+      <c r="D1302" s="2">
+        <v>45232</v>
       </c>
       <c r="E1302">
         <v>183000</v>
@@ -22828,8 +22684,8 @@
       <c r="C1303" t="s">
         <v>50</v>
       </c>
-      <c r="D1303" t="s">
-        <v>84</v>
+      <c r="D1303" s="2">
+        <v>45324</v>
       </c>
       <c r="E1303">
         <v>336000</v>
@@ -22845,8 +22701,8 @@
       <c r="C1304" t="s">
         <v>50</v>
       </c>
-      <c r="D1304" t="s">
-        <v>85</v>
+      <c r="D1304" s="2">
+        <v>45418</v>
       </c>
       <c r="E1304">
         <v>279000</v>
@@ -22862,8 +22718,8 @@
       <c r="C1305" t="s">
         <v>50</v>
       </c>
-      <c r="D1305" t="s">
-        <v>86</v>
+      <c r="D1305" s="2">
+        <v>45506</v>
       </c>
       <c r="E1305">
         <v>413000</v>
@@ -22879,8 +22735,8 @@
       <c r="C1306" t="s">
         <v>50</v>
       </c>
-      <c r="D1306" t="s">
-        <v>87</v>
+      <c r="D1306" s="2">
+        <v>45600</v>
       </c>
       <c r="E1306">
         <v>371000</v>
@@ -22896,8 +22752,8 @@
       <c r="C1307" t="s">
         <v>50</v>
       </c>
-      <c r="D1307" t="s">
-        <v>88</v>
+      <c r="D1307" s="2">
+        <v>45695</v>
       </c>
       <c r="E1307">
         <v>572000</v>
@@ -22913,8 +22769,8 @@
       <c r="C1308" t="s">
         <v>50</v>
       </c>
-      <c r="D1308" t="s">
-        <v>89</v>
+      <c r="D1308" s="2">
+        <v>45779</v>
       </c>
       <c r="E1308">
         <v>526000</v>
@@ -22930,8 +22786,8 @@
       <c r="C1309" t="s">
         <v>50</v>
       </c>
-      <c r="D1309" t="s">
-        <v>90</v>
+      <c r="D1309" s="2">
+        <v>45874</v>
       </c>
       <c r="E1309">
         <v>402000</v>
@@ -22947,8 +22803,8 @@
       <c r="C1310" t="s">
         <v>50</v>
       </c>
-      <c r="D1310" t="s">
-        <v>91</v>
+      <c r="D1310" s="2">
+        <v>45965</v>
       </c>
       <c r="E1310">
         <v>215000</v>
@@ -22964,8 +22820,8 @@
       <c r="C1311" t="s">
         <v>50</v>
       </c>
-      <c r="D1311" t="s">
-        <v>92</v>
+      <c r="D1311" s="2">
+        <v>46059</v>
       </c>
       <c r="E1311">
         <v>17000</v>
@@ -22981,8 +22837,8 @@
       <c r="C1312" t="s">
         <v>51</v>
       </c>
-      <c r="D1312" t="s">
-        <v>93</v>
+      <c r="D1312" s="2">
+        <v>45464</v>
       </c>
       <c r="E1312">
         <v>0</v>
@@ -22998,8 +22854,8 @@
       <c r="C1313" t="s">
         <v>51</v>
       </c>
-      <c r="D1313" t="s">
-        <v>94</v>
+      <c r="D1313" s="2">
+        <v>45558</v>
       </c>
       <c r="E1313">
         <v>162000</v>
@@ -23015,8 +22871,8 @@
       <c r="C1314" t="s">
         <v>51</v>
       </c>
-      <c r="D1314" t="s">
-        <v>95</v>
+      <c r="D1314" s="2">
+        <v>45645</v>
       </c>
       <c r="E1314">
         <v>207000</v>
@@ -23032,8 +22888,8 @@
       <c r="C1315" t="s">
         <v>51</v>
       </c>
-      <c r="D1315" t="s">
-        <v>96</v>
+      <c r="D1315" s="2">
+        <v>45736</v>
       </c>
       <c r="E1315">
         <v>155000</v>
@@ -23049,8 +22905,8 @@
       <c r="C1316" t="s">
         <v>51</v>
       </c>
-      <c r="D1316" t="s">
-        <v>97</v>
+      <c r="D1316" s="2">
+        <v>45826</v>
       </c>
       <c r="E1316">
         <v>1338000</v>
@@ -23066,8 +22922,8 @@
       <c r="C1317" t="s">
         <v>51</v>
       </c>
-      <c r="D1317" t="s">
-        <v>98</v>
+      <c r="D1317" s="2">
+        <v>45919</v>
       </c>
       <c r="E1317">
         <v>1971000</v>
@@ -23083,8 +22939,8 @@
       <c r="C1318" t="s">
         <v>51</v>
       </c>
-      <c r="D1318" t="s">
-        <v>99</v>
+      <c r="D1318" s="2">
+        <v>46014</v>
       </c>
       <c r="E1318">
         <v>246000</v>

</xml_diff>